<commit_message>
Switch TEA inputs to 551 scale datasets
Point tea_ccs, tea_co2_portion, and tea_scale_up_price_models at the
Pyrolysis_551 stream/APEA files (CO2 portion at scale 300, galik folders
renamed) and regenerate the CCS/scale-up figures and CO2 result sheets.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Figure/TEA_summary_CCS.xlsx
+++ b/Figure/TEA_summary_CCS.xlsx
@@ -462,19 +462,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>384.2928854614783</v>
+        <v>428.6643822549371</v>
       </c>
       <c r="C2" t="n">
-        <v>391.7419768550133</v>
+        <v>436.0757725222338</v>
       </c>
       <c r="D2" t="n">
-        <v>399.1910682485483</v>
+        <v>443.4871627895304</v>
       </c>
       <c r="E2" t="n">
-        <v>406.6401596420832</v>
+        <v>450.898553056827</v>
       </c>
       <c r="F2" t="n">
-        <v>414.0892510356182</v>
+        <v>458.3099433241238</v>
       </c>
     </row>
     <row r="3">
@@ -484,19 +484,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>73.02621018566622</v>
+        <v>72.96704634612149</v>
       </c>
       <c r="C3" t="n">
-        <v>73.02621018566622</v>
+        <v>72.96704634612149</v>
       </c>
       <c r="D3" t="n">
-        <v>73.02621018566622</v>
+        <v>72.96704634612149</v>
       </c>
       <c r="E3" t="n">
-        <v>73.02621018566622</v>
+        <v>72.96704634612149</v>
       </c>
       <c r="F3" t="n">
-        <v>73.02621018566622</v>
+        <v>72.96704634612149</v>
       </c>
     </row>
     <row r="4">
@@ -506,19 +506,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>32.8007149915544</v>
+        <v>37.7160153684562</v>
       </c>
       <c r="C4" t="n">
-        <v>38.05470124644303</v>
+        <v>39.47548086935472</v>
       </c>
       <c r="D4" t="n">
-        <v>49.35810709068012</v>
+        <v>41.23494637025323</v>
       </c>
       <c r="E4" t="n">
-        <v>60.66151293491721</v>
+        <v>51.01928719573782</v>
       </c>
       <c r="F4" t="n">
-        <v>71.96491877915429</v>
+        <v>62.26548456874759</v>
       </c>
     </row>
     <row r="5">
@@ -528,19 +528,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.8</v>
+        <v>2.04</v>
       </c>
       <c r="C5" t="n">
-        <v>2.8</v>
+        <v>2.04</v>
       </c>
       <c r="D5" t="n">
-        <v>2.8</v>
+        <v>2.04</v>
       </c>
       <c r="E5" t="n">
-        <v>2.8</v>
+        <v>2.04</v>
       </c>
       <c r="F5" t="n">
-        <v>2.8</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="6">
@@ -550,19 +550,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5.39</v>
+        <v>6.23</v>
       </c>
       <c r="C6" t="n">
-        <v>5.39</v>
+        <v>6.23</v>
       </c>
       <c r="D6" t="n">
-        <v>5.39</v>
+        <v>6.23</v>
       </c>
       <c r="E6" t="n">
-        <v>5.39</v>
+        <v>6.23</v>
       </c>
       <c r="F6" t="n">
-        <v>5.39</v>
+        <v>6.23</v>
       </c>
     </row>
     <row r="7">
@@ -572,19 +572,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.7</v>
+        <v>0.51</v>
       </c>
       <c r="C7" t="n">
-        <v>0.7</v>
+        <v>0.51</v>
       </c>
       <c r="D7" t="n">
-        <v>0.7</v>
+        <v>0.51</v>
       </c>
       <c r="E7" t="n">
-        <v>0.7</v>
+        <v>0.51</v>
       </c>
       <c r="F7" t="n">
-        <v>0.7</v>
+        <v>0.51</v>
       </c>
     </row>
     <row r="8">
@@ -594,19 +594,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4.095</v>
+        <v>4.135</v>
       </c>
       <c r="C8" t="n">
-        <v>4.095</v>
+        <v>4.135</v>
       </c>
       <c r="D8" t="n">
-        <v>4.095</v>
+        <v>4.135</v>
       </c>
       <c r="E8" t="n">
-        <v>4.095</v>
+        <v>4.135</v>
       </c>
       <c r="F8" t="n">
-        <v>4.095</v>
+        <v>4.135</v>
       </c>
     </row>
     <row r="9">
@@ -616,19 +616,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9.3711</v>
+        <v>9.754</v>
       </c>
       <c r="C9" t="n">
-        <v>9.3711</v>
+        <v>9.754</v>
       </c>
       <c r="D9" t="n">
-        <v>9.3711</v>
+        <v>9.754</v>
       </c>
       <c r="E9" t="n">
-        <v>9.3711</v>
+        <v>9.754</v>
       </c>
       <c r="F9" t="n">
-        <v>9.3711</v>
+        <v>9.754</v>
       </c>
     </row>
     <row r="10">
@@ -638,19 +638,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>55.81858984852092</v>
+        <v>62.26355532714233</v>
       </c>
       <c r="C10" t="n">
-        <v>56.90057130841852</v>
+        <v>63.34006069372169</v>
       </c>
       <c r="D10" t="n">
-        <v>57.98255276831615</v>
+        <v>64.41656606030107</v>
       </c>
       <c r="E10" t="n">
-        <v>59.06453422821375</v>
+        <v>65.49307142688043</v>
       </c>
       <c r="F10" t="n">
-        <v>60.14651568811136</v>
+        <v>66.5695767934598</v>
       </c>
     </row>
     <row r="11">
@@ -660,19 +660,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-103.2051895794363</v>
+        <v>-105.7117597047233</v>
       </c>
       <c r="C11" t="n">
-        <v>-103.2051895794363</v>
+        <v>-105.7117597047233</v>
       </c>
       <c r="D11" t="n">
-        <v>-103.2051895794363</v>
+        <v>-105.7117597047233</v>
       </c>
       <c r="E11" t="n">
-        <v>-103.2051895794363</v>
+        <v>-105.7117597047233</v>
       </c>
       <c r="F11" t="n">
-        <v>-103.2051895794363</v>
+        <v>-105.7117597047233</v>
       </c>
     </row>
   </sheetData>

</xml_diff>